<commit_message>
Updated code to get excel response in object form using okhttp.
</commit_message>
<xml_diff>
--- a/src/main/resources/Demo.xlsx
+++ b/src/main/resources/Demo.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="2">
   <si>
     <t>New Course</t>
   </si>
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BE27858-AAF3-4E86-BA69-820BD90AC0C3}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="10.54296875"/>
@@ -436,6 +436,14 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>